<commit_message>
fix: mobile layout AC summary
</commit_message>
<xml_diff>
--- a/src/data/QMO26-SAS.xlsx
+++ b/src/data/QMO26-SAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Haruj\gear-motor-app\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{628FBACA-3299-4AF7-8921-06C1F2216395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AAE935-E063-4063-8BB0-52C73CD337D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -874,6 +874,15 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -896,15 +905,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1228,8 +1228,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="142874" y="14967014"/>
-          <a:ext cx="8216300" cy="3140340"/>
+          <a:off x="142874" y="15142329"/>
+          <a:ext cx="8193983" cy="3152764"/>
           <a:chOff x="152400" y="10250543"/>
           <a:chExt cx="7652668" cy="2826224"/>
         </a:xfrm>
@@ -1288,7 +1288,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1301,7 +1301,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1314,7 +1314,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1327,7 +1327,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1340,7 +1340,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1354,7 +1354,7 @@
               <a:defRPr sz="1000"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1369,7 +1369,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1383,7 +1383,7 @@
               <a:defRPr sz="1000"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1399,7 +1399,7 @@
               <a:defRPr sz="1000"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1415,7 +1415,7 @@
               <a:defRPr sz="1000"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1431,7 +1431,7 @@
               <a:defRPr sz="1000"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -1446,7 +1446,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1459,7 +1459,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1472,7 +1472,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1485,7 +1485,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -2105,8 +2105,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8517209" y="2143125"/>
-          <a:ext cx="4202908" cy="1301750"/>
+          <a:off x="8488910" y="2154168"/>
+          <a:ext cx="4212801" cy="1321077"/>
           <a:chOff x="8028215" y="2589250"/>
           <a:chExt cx="3625038" cy="824781"/>
         </a:xfrm>
@@ -2166,7 +2166,7 @@
               <a:defRPr sz="1000"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1300" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:rPr lang="en-US" sz="1300" b="1" i="0" u="none" strike="noStrike" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -2181,7 +2181,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="1050" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -2194,7 +2194,7 @@
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
             </a:pPr>
-            <a:endParaRPr lang="en-US" sz="1050" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:endParaRPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike" baseline="0">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -2240,15 +2240,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>103190</xdr:colOff>
+      <xdr:colOff>462103</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>174432</xdr:rowOff>
+      <xdr:rowOff>146823</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>373064</xdr:colOff>
+      <xdr:colOff>731977</xdr:colOff>
       <xdr:row>56</xdr:row>
-      <xdr:rowOff>150495</xdr:rowOff>
+      <xdr:rowOff>122886</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2274,8 +2274,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="10697107" y="16081182"/>
-          <a:ext cx="1402291" cy="801563"/>
+          <a:off x="9582175" y="15598490"/>
+          <a:ext cx="1401831" cy="822729"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2740,9 +2740,9 @@
     </row>
     <row r="12" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
-      <c r="B12" s="90"/>
-      <c r="C12" s="90"/>
-      <c r="D12" s="90"/>
+      <c r="B12" s="82"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
       <c r="E12" s="10"/>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
@@ -2791,14 +2791,14 @@
       <c r="C16" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="91" t="s">
+      <c r="D16" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="E16" s="91"/>
-      <c r="F16" s="91" t="s">
+      <c r="E16" s="83"/>
+      <c r="F16" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="G16" s="92"/>
+      <c r="G16" s="84"/>
       <c r="H16" s="65" t="s">
         <v>3</v>
       </c>
@@ -2813,14 +2813,14 @@
       <c r="C17" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="87" t="s">
+      <c r="D17" s="90" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="87"/>
-      <c r="F17" s="88" t="s">
+      <c r="E17" s="90"/>
+      <c r="F17" s="91" t="s">
         <v>34</v>
       </c>
-      <c r="G17" s="88"/>
+      <c r="G17" s="91"/>
       <c r="H17" s="24" t="s">
         <v>32</v>
       </c>
@@ -2842,11 +2842,11 @@
       <c r="B19" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="89" t="s">
+      <c r="C19" s="92" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="89"/>
-      <c r="E19" s="89"/>
+      <c r="D19" s="92"/>
+      <c r="E19" s="92"/>
       <c r="F19" s="63" t="s">
         <v>4</v>
       </c>
@@ -3181,9 +3181,9 @@
     <row r="48" spans="1:10" s="31" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="23"/>
       <c r="B48" s="29"/>
-      <c r="C48" s="84"/>
-      <c r="D48" s="85"/>
-      <c r="E48" s="86"/>
+      <c r="C48" s="87"/>
+      <c r="D48" s="88"/>
+      <c r="E48" s="89"/>
       <c r="F48" s="30"/>
       <c r="G48" s="41"/>
       <c r="H48" s="56"/>
@@ -3243,11 +3243,11 @@
       <c r="D52" s="15"/>
       <c r="E52" s="15"/>
       <c r="F52" s="34"/>
-      <c r="G52" s="83" t="str">
+      <c r="G52" s="86" t="str">
         <f>"("&amp;BAHTTEXT(H$51)&amp;")"</f>
         <v>(ศูนย์บาทถ้วน)</v>
       </c>
-      <c r="H52" s="83"/>
+      <c r="H52" s="86"/>
     </row>
     <row r="53" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="35"/>
@@ -3291,8 +3291,8 @@
       <c r="G58" s="39"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D61" s="82"/>
-      <c r="E61" s="82"/>
+      <c r="D61" s="85"/>
+      <c r="E61" s="85"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
Update PDF , จอ
</commit_message>
<xml_diff>
--- a/src/data/QMO26-SAS.xlsx
+++ b/src/data/QMO26-SAS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr checkCompatibility="1" autoCompressPictures="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Haruj\gear-motor-app\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AAE935-E063-4063-8BB0-52C73CD337D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D78E196-D747-491E-AFF1-A7D4011385F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>DESCRIPTION</t>
   </si>
@@ -165,9 +165,6 @@
     <t>18 Months</t>
   </si>
   <si>
-    <t>Within 30-45 days</t>
-  </si>
-  <si>
     <t>QMO26-SAS-001</t>
   </si>
   <si>
@@ -175,6 +172,118 @@
   </si>
   <si>
     <t>AC Gear Motor</t>
+  </si>
+  <si>
+    <t>QUOTATION
+ใบเสนอราคา</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LINE ID: @synergy.as  </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+                                                                                                                                                                           ___________________________________________                                </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Mr. Chottanin A. (CA) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+TRANSMISSION PRODUCT MANAGER : 081-921-6225
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+______________________________________         
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">To confirm this quotation, sign here and return: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">                                                                  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>Date   ......./......../...........</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">                                       Approve By</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Trebuchet MS"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">                                                                       </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mr.Traiwit Luengthong</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">                              SALE MANAGER</t>
+    </r>
+  </si>
+  <si>
+    <t>On the table</t>
   </si>
 </sst>
 </file>
@@ -190,7 +299,7 @@
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="168" formatCode="[$-1070000]d/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="39" x14ac:knownFonts="1">
+  <fonts count="41" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -317,13 +426,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Trebuchet MS"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Trebuchet MS"/>
@@ -345,14 +447,6 @@
     <font>
       <b/>
       <sz val="9"/>
-      <color theme="1"/>
-      <name val="Trebuchet MS"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="10"/>
       <color theme="1"/>
       <name val="Trebuchet MS"/>
       <family val="2"/>
@@ -434,6 +528,33 @@
     <font>
       <sz val="12"/>
       <color rgb="FF0070C0"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color rgb="FF0070C0"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
@@ -663,9 +784,9 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="32" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="99">
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -741,24 +862,18 @@
     <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="167" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="44" fontId="24" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -768,7 +883,7 @@
     <xf numFmtId="165" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -777,7 +892,7 @@
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -793,13 +908,13 @@
     <xf numFmtId="43" fontId="18" fillId="0" borderId="5" xfId="108" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="31" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="18" fillId="0" borderId="1" xfId="112" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -814,10 +929,10 @@
     <xf numFmtId="1" fontId="18" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -835,40 +950,40 @@
     <xf numFmtId="44" fontId="20" fillId="0" borderId="0" xfId="112" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="34" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="32" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="36" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="31" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="38" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="37" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="27" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="35" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="33" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -883,19 +998,16 @@
     <xf numFmtId="165" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="29" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="27" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="37" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="37" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="35" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="37" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -906,6 +1018,33 @@
     </xf>
     <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="113">
@@ -1108,16 +1247,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>465066</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3327167</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>15871</xdr:rowOff>
+      <xdr:rowOff>282755</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1551201</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>136520</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>271998</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>16882</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1134,8 +1273,8 @@
       </xdr:nvSpPr>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="8815917" y="15871"/>
-          <a:ext cx="2995083" cy="1025524"/>
+          <a:off x="6391732" y="282755"/>
+          <a:ext cx="3000338" cy="1022533"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1168,29 +1307,6 @@
           <a:pPr algn="r" rtl="0">
             <a:defRPr sz="1000"/>
           </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="2400" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="3B5E91"/>
-              </a:solidFill>
-              <a:latin typeface="Trebuchet MS"/>
-            </a:rPr>
-            <a:t>QUOTATION</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="r" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="th-TH" sz="1800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="3B5E91"/>
-              </a:solidFill>
-              <a:latin typeface="Trebuchet MS"/>
-            </a:rPr>
-            <a:t>ใบเสนอราคา</a:t>
-          </a:r>
           <a:endParaRPr lang="en-US" sz="1800" b="1" i="0" u="none" strike="noStrike" baseline="0">
             <a:solidFill>
               <a:srgbClr val="3B5E91"/>
@@ -1204,542 +1320,82 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>142874</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>12764</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1041152</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>31169</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>2367949</xdr:colOff>
-      <xdr:row>67</xdr:row>
-      <xdr:rowOff>73354</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>164683</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>121625</xdr:rowOff>
     </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="3" name="Group 2">
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Text Box 18">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="142874" y="15142329"/>
-          <a:ext cx="8193983" cy="3152764"/>
-          <a:chOff x="152400" y="10250543"/>
-          <a:chExt cx="7652668" cy="2826224"/>
+          <a:off x="4105717" y="13228126"/>
+          <a:ext cx="4396792" cy="2842122"/>
         </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="4" name="Text Box 18">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr txBox="1">
-            <a:spLocks noChangeArrowheads="1"/>
-          </xdr:cNvSpPr>
-        </xdr:nvSpPr>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="152400" y="10517715"/>
-            <a:ext cx="3175000" cy="2559052"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65">
-                    <a:alpha val="0"/>
-                  </a:srgbClr>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" upright="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
               </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
               </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>______________________________________         </a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>To confirm this quotation, sign here and return:  </a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t> </a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t> </a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>             Date   ......./......../...........</a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="5" name="Text Box 18">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr txBox="1">
-            <a:spLocks noChangeArrowheads="1"/>
-          </xdr:cNvSpPr>
-        </xdr:nvSpPr>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="3698739" y="10250543"/>
-            <a:ext cx="4106329" cy="2547756"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65">
-                    <a:alpha val="0"/>
-                  </a:srgbClr>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" upright="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>                                                                                                                         ____________________________________________                                                                                                                                                                                                                                                      </a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:br>
-              <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-            </a:br>
-            <a:r>
-              <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>Mr. Chottanin A. (CA) </a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>TRANSMISSION PRODUCT MANAGER</a:t>
-            </a:r>
-            <a:br>
-              <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-            </a:br>
-            <a:r>
-              <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>081-921-6225</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-    </xdr:grpSp>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" upright="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
@@ -1788,309 +1444,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>615684</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>103187</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2651969</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>107013</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1451768</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Text Box 18">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="9100872" y="15382875"/>
-          <a:ext cx="3272896" cy="2341563"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65">
-                  <a:alpha val="0"/>
-                </a:srgbClr>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="900">
-              <a:effectLst/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>                                                                                                                         </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>                                                                                                                 </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>                                                                                                                                                 </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Approve By</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>                                                                                                                                       </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Mr.Traiwit Luengthong </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>                                                                                                                                               </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>SALE MANAGER</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>151084</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>111125</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>20117</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>472464</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>79375</xdr:rowOff>
+      <xdr:rowOff>42564</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2105,10 +1468,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8488910" y="2154168"/>
-          <a:ext cx="4212801" cy="1321077"/>
-          <a:chOff x="8028215" y="2589250"/>
-          <a:chExt cx="3625038" cy="824781"/>
+          <a:off x="5716534" y="1588680"/>
+          <a:ext cx="3876002" cy="1849754"/>
+          <a:chOff x="5801015" y="2259184"/>
+          <a:chExt cx="3335229" cy="1154847"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:sp macro="" textlink="">
@@ -2126,7 +1489,7 @@
         </xdr:nvSpPr>
         <xdr:spPr bwMode="auto">
           <a:xfrm>
-            <a:off x="9348694" y="2885454"/>
+            <a:off x="5801015" y="2259184"/>
             <a:ext cx="2304559" cy="333376"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
@@ -2161,35 +1524,6 @@
         <xdr:txBody>
           <a:bodyPr vertOverflow="clip" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" upright="1"/>
           <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1300" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-              </a:rPr>
-              <a:t>LINE ID: @synergy.as                                                                                                                                                                                                                                                            </a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="l" rtl="0">
-              <a:defRPr sz="1000"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="1050" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" pitchFamily="34" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
           <a:p>
             <a:pPr algn="l" rtl="0">
               <a:defRPr sz="1000"/>
@@ -2239,16 +1573,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>462103</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>146823</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>719783</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>184058</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>731977</xdr:colOff>
+      <xdr:colOff>677109</xdr:colOff>
       <xdr:row>56</xdr:row>
-      <xdr:rowOff>122886</xdr:rowOff>
+      <xdr:rowOff>113683</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2274,8 +1608,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="9582175" y="15598490"/>
-          <a:ext cx="1401831" cy="822729"/>
+          <a:off x="9057609" y="15313623"/>
+          <a:ext cx="1871529" cy="1098393"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2587,7 +1921,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.1796875" style="3" customWidth="1"/>
@@ -2612,7 +1946,10 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="G1" s="95" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="94"/>
     </row>
     <row r="2" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
@@ -2638,7 +1975,7 @@
         <v>9</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -2653,7 +1990,7 @@
       <c r="G4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="50">
+      <c r="H4" s="48">
         <f ca="1">TODAY()</f>
         <v>46084</v>
       </c>
@@ -2670,7 +2007,7 @@
       <c r="G5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="51" t="s">
+      <c r="H5" s="49" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2700,7 +2037,7 @@
       <c r="G7" s="5"/>
     </row>
     <row r="8" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="47" t="s">
         <v>27</v>
       </c>
       <c r="B8" s="11"/>
@@ -2712,48 +2049,52 @@
     </row>
     <row r="9" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4"/>
-      <c r="B9" s="46"/>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
+      <c r="B9" s="44"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
       <c r="E9" s="12"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
     </row>
     <row r="10" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
-      <c r="B10" s="80"/>
-      <c r="C10" s="80"/>
-      <c r="D10" s="80"/>
-      <c r="E10" s="80"/>
+      <c r="B10" s="78"/>
+      <c r="C10" s="78"/>
+      <c r="D10" s="78"/>
+      <c r="E10" s="78"/>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="M10"/>
     </row>
     <row r="11" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
-      <c r="B11" s="81"/>
-      <c r="C11" s="81"/>
-      <c r="D11" s="81"/>
-      <c r="E11" s="47"/>
+      <c r="B11" s="79"/>
+      <c r="C11" s="79"/>
+      <c r="D11" s="79"/>
+      <c r="E11" s="45"/>
       <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
+      <c r="G11" s="97" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" s="96"/>
     </row>
     <row r="12" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
-      <c r="B12" s="82"/>
-      <c r="C12" s="82"/>
-      <c r="D12" s="82"/>
+      <c r="B12" s="80"/>
+      <c r="C12" s="80"/>
+      <c r="D12" s="80"/>
       <c r="E12" s="10"/>
       <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
+      <c r="G12" s="96"/>
+      <c r="H12" s="96"/>
     </row>
     <row r="13" spans="1:13" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="78"/>
-      <c r="C13" s="79"/>
-      <c r="D13" s="79"/>
+      <c r="B13" s="76"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
       <c r="E13" s="10"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
@@ -2762,7 +2103,7 @@
       <c r="A14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="61"/>
+      <c r="B14" s="59"/>
       <c r="C14" s="10"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
@@ -2773,7 +2114,7 @@
       <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="46"/>
       <c r="C15" s="12"/>
       <c r="D15" s="13"/>
       <c r="E15" s="13"/>
@@ -2782,45 +2123,45 @@
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:13" s="16" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="64" t="s">
+      <c r="A16" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="64" t="s">
+      <c r="B16" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="64" t="s">
+      <c r="C16" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="83" t="s">
+      <c r="D16" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="E16" s="83"/>
-      <c r="F16" s="83" t="s">
+      <c r="E16" s="81"/>
+      <c r="F16" s="81" t="s">
         <v>2</v>
       </c>
-      <c r="G16" s="84"/>
-      <c r="H16" s="65" t="s">
+      <c r="G16" s="82"/>
+      <c r="H16" s="63" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:10" s="17" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="58" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="45" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="90" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="90"/>
-      <c r="F17" s="91" t="s">
-        <v>34</v>
-      </c>
-      <c r="G17" s="91"/>
+      <c r="E17" s="87"/>
+      <c r="F17" s="88" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" s="88"/>
       <c r="H17" s="24" t="s">
         <v>32</v>
       </c>
@@ -2836,40 +2177,40 @@
       <c r="H18" s="22"/>
     </row>
     <row r="19" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="62" t="s">
+      <c r="A19" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="62" t="s">
+      <c r="B19" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="92" t="s">
+      <c r="C19" s="89" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="92"/>
-      <c r="E19" s="92"/>
-      <c r="F19" s="63" t="s">
+      <c r="D19" s="89"/>
+      <c r="E19" s="89"/>
+      <c r="F19" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="G19" s="63" t="s">
+      <c r="G19" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="H19" s="63" t="s">
+      <c r="H19" s="61" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:10" s="27" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="59">
+      <c r="A20" s="57">
         <v>1</v>
       </c>
       <c r="B20" s="24"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="58"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="56"/>
       <c r="F20" s="25">
         <v>1</v>
       </c>
-      <c r="G20" s="56"/>
-      <c r="H20" s="56">
+      <c r="G20" s="54"/>
+      <c r="H20" s="54">
         <f>G20*F20</f>
         <v>0</v>
       </c>
@@ -2878,315 +2219,315 @@
     <row r="21" spans="1:10" s="27" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="24"/>
       <c r="B21" s="24"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="43"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="41"/>
       <c r="F21" s="25"/>
-      <c r="G21" s="68"/>
-      <c r="H21" s="56"/>
+      <c r="G21" s="66"/>
+      <c r="H21" s="54"/>
       <c r="I21" s="26"/>
     </row>
     <row r="22" spans="1:10" s="27" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="24"/>
       <c r="B22" s="24"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="43"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="41"/>
       <c r="F22" s="25"/>
-      <c r="G22" s="56"/>
-      <c r="H22" s="56">
+      <c r="G22" s="54"/>
+      <c r="H22" s="54">
         <f t="shared" ref="H22:H24" si="0">G22*F22</f>
         <v>0</v>
       </c>
       <c r="I22" s="26"/>
     </row>
     <row r="23" spans="1:10" s="27" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="59"/>
+      <c r="A23" s="57"/>
       <c r="B23" s="24"/>
-      <c r="C23" s="73"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="58"/>
+      <c r="C23" s="71"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="56"/>
       <c r="F23" s="25"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
+      <c r="G23" s="54"/>
+      <c r="H23" s="54"/>
       <c r="I23" s="26"/>
     </row>
     <row r="24" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="24"/>
       <c r="B24" s="24"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="42"/>
-      <c r="E24" s="43"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="41"/>
       <c r="F24" s="25"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="56">
+      <c r="G24" s="66"/>
+      <c r="H24" s="54">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J24" s="28"/>
     </row>
     <row r="25" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="59"/>
+      <c r="A25" s="57"/>
       <c r="B25" s="24"/>
-      <c r="C25" s="70"/>
-      <c r="D25" s="57"/>
-      <c r="E25" s="58"/>
+      <c r="C25" s="68"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="56"/>
       <c r="F25" s="25"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="54"/>
       <c r="J25" s="28"/>
     </row>
     <row r="26" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="24"/>
       <c r="B26" s="24"/>
-      <c r="C26" s="41"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="43"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="25"/>
-      <c r="G26" s="67"/>
-      <c r="H26" s="56"/>
-      <c r="J26" s="66"/>
+      <c r="G26" s="65"/>
+      <c r="H26" s="54"/>
+      <c r="J26" s="64"/>
     </row>
     <row r="27" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="24"/>
       <c r="B27" s="24"/>
-      <c r="C27" s="73"/>
-      <c r="D27" s="42"/>
-      <c r="E27" s="43"/>
+      <c r="C27" s="71"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="41"/>
       <c r="F27" s="25"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="56"/>
-      <c r="J27" s="66"/>
+      <c r="G27" s="65"/>
+      <c r="H27" s="54"/>
+      <c r="J27" s="64"/>
     </row>
     <row r="28" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="24"/>
       <c r="B28" s="24"/>
-      <c r="C28" s="73"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="43"/>
+      <c r="C28" s="71"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="41"/>
       <c r="F28" s="25"/>
-      <c r="G28" s="67"/>
-      <c r="H28" s="56"/>
-      <c r="J28" s="66"/>
+      <c r="G28" s="65"/>
+      <c r="H28" s="54"/>
+      <c r="J28" s="64"/>
     </row>
     <row r="29" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="24"/>
       <c r="B29" s="24"/>
-      <c r="C29" s="73"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="43"/>
+      <c r="C29" s="71"/>
+      <c r="D29" s="40"/>
+      <c r="E29" s="41"/>
       <c r="F29" s="25"/>
-      <c r="G29" s="56"/>
-      <c r="H29" s="56"/>
-      <c r="J29" s="66"/>
+      <c r="G29" s="54"/>
+      <c r="H29" s="54"/>
+      <c r="J29" s="64"/>
     </row>
     <row r="30" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="59"/>
+      <c r="A30" s="57"/>
       <c r="B30" s="24"/>
-      <c r="C30" s="41"/>
-      <c r="D30" s="57"/>
-      <c r="E30" s="58"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="56"/>
       <c r="F30" s="25"/>
-      <c r="G30" s="56"/>
-      <c r="H30" s="56"/>
-      <c r="J30" s="66"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="54"/>
+      <c r="J30" s="64"/>
     </row>
     <row r="31" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="24"/>
       <c r="B31" s="24"/>
-      <c r="C31" s="41"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="43"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="40"/>
+      <c r="E31" s="41"/>
       <c r="F31" s="25"/>
-      <c r="G31" s="68"/>
-      <c r="H31" s="56"/>
-      <c r="J31" s="66"/>
+      <c r="G31" s="66"/>
+      <c r="H31" s="54"/>
+      <c r="J31" s="64"/>
     </row>
     <row r="32" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="59"/>
+      <c r="A32" s="57"/>
       <c r="B32" s="24"/>
-      <c r="C32" s="70"/>
-      <c r="D32" s="57"/>
-      <c r="E32" s="58"/>
+      <c r="C32" s="68"/>
+      <c r="D32" s="55"/>
+      <c r="E32" s="56"/>
       <c r="F32" s="25"/>
-      <c r="G32" s="56"/>
-      <c r="H32" s="56"/>
-      <c r="J32" s="66"/>
+      <c r="G32" s="54"/>
+      <c r="H32" s="54"/>
+      <c r="J32" s="64"/>
     </row>
     <row r="33" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="24"/>
       <c r="B33" s="24"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="43"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="41"/>
       <c r="F33" s="25"/>
-      <c r="G33" s="67"/>
-      <c r="H33" s="56"/>
-      <c r="J33" s="66"/>
+      <c r="G33" s="65"/>
+      <c r="H33" s="54"/>
+      <c r="J33" s="64"/>
     </row>
     <row r="34" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="24"/>
       <c r="B34" s="24"/>
-      <c r="C34" s="69"/>
-      <c r="D34" s="42"/>
-      <c r="E34" s="43"/>
+      <c r="C34" s="67"/>
+      <c r="D34" s="40"/>
+      <c r="E34" s="41"/>
       <c r="F34" s="25"/>
-      <c r="G34" s="67"/>
-      <c r="H34" s="56"/>
-      <c r="J34" s="66"/>
+      <c r="G34" s="65"/>
+      <c r="H34" s="54"/>
+      <c r="J34" s="64"/>
     </row>
     <row r="35" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="24"/>
       <c r="B35" s="24"/>
-      <c r="C35" s="41"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="43"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="40"/>
+      <c r="E35" s="41"/>
       <c r="F35" s="25"/>
-      <c r="G35" s="67"/>
-      <c r="H35" s="56"/>
-      <c r="J35" s="66"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="54"/>
+      <c r="J35" s="64"/>
     </row>
     <row r="36" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="24"/>
       <c r="B36" s="24"/>
-      <c r="C36" s="69"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
+      <c r="C36" s="67"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="41"/>
       <c r="F36" s="25"/>
-      <c r="G36" s="67"/>
-      <c r="H36" s="56"/>
-      <c r="J36" s="66"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="54"/>
+      <c r="J36" s="64"/>
     </row>
     <row r="37" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="24"/>
       <c r="B37" s="24"/>
-      <c r="C37" s="41"/>
-      <c r="D37" s="42"/>
-      <c r="E37" s="43"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="40"/>
+      <c r="E37" s="41"/>
       <c r="F37" s="25"/>
-      <c r="G37" s="67"/>
-      <c r="H37" s="56"/>
-      <c r="J37" s="66"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="54"/>
+      <c r="J37" s="64"/>
     </row>
     <row r="38" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="24"/>
       <c r="B38" s="24"/>
-      <c r="C38" s="41"/>
-      <c r="D38" s="42"/>
-      <c r="E38" s="43"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="40"/>
+      <c r="E38" s="41"/>
       <c r="F38" s="25"/>
-      <c r="G38" s="56"/>
-      <c r="H38" s="56"/>
+      <c r="G38" s="54"/>
+      <c r="H38" s="54"/>
       <c r="J38" s="28"/>
     </row>
     <row r="39" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="59"/>
+      <c r="A39" s="57"/>
       <c r="B39" s="24"/>
-      <c r="C39" s="41"/>
+      <c r="C39" s="39"/>
       <c r="D39"/>
       <c r="E39"/>
       <c r="F39" s="25"/>
-      <c r="G39" s="56"/>
-      <c r="H39" s="56"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="54"/>
       <c r="J39" s="28"/>
     </row>
     <row r="40" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="24"/>
       <c r="B40" s="24"/>
-      <c r="C40" s="41"/>
-      <c r="D40" s="42"/>
-      <c r="E40" s="43"/>
+      <c r="C40" s="39"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="41"/>
       <c r="F40" s="25"/>
-      <c r="G40" s="68"/>
-      <c r="H40" s="56"/>
+      <c r="G40" s="66"/>
+      <c r="H40" s="54"/>
       <c r="J40" s="28"/>
     </row>
     <row r="41" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="59"/>
+      <c r="A41" s="57"/>
       <c r="B41" s="24"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="57"/>
-      <c r="E41" s="58"/>
+      <c r="C41" s="68"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="56"/>
       <c r="F41" s="25"/>
-      <c r="G41" s="56"/>
-      <c r="H41" s="56"/>
+      <c r="G41" s="54"/>
+      <c r="H41" s="54"/>
       <c r="J41" s="28"/>
     </row>
     <row r="42" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="24"/>
       <c r="B42" s="24"/>
-      <c r="C42" s="41"/>
-      <c r="D42" s="42"/>
-      <c r="E42" s="43"/>
+      <c r="C42" s="39"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="41"/>
       <c r="F42" s="25"/>
-      <c r="G42" s="67"/>
-      <c r="H42" s="56"/>
+      <c r="G42" s="65"/>
+      <c r="H42" s="54"/>
       <c r="J42" s="28"/>
     </row>
     <row r="43" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="24"/>
       <c r="B43" s="24"/>
-      <c r="C43" s="70"/>
-      <c r="D43" s="57"/>
-      <c r="E43" s="58"/>
+      <c r="C43" s="68"/>
+      <c r="D43" s="55"/>
+      <c r="E43" s="56"/>
       <c r="F43" s="25"/>
-      <c r="G43" s="67"/>
-      <c r="H43" s="56"/>
+      <c r="G43" s="65"/>
+      <c r="H43" s="54"/>
       <c r="J43" s="28"/>
     </row>
     <row r="44" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="59"/>
+      <c r="A44" s="57"/>
       <c r="B44" s="24"/>
-      <c r="C44" s="41"/>
-      <c r="D44" s="42"/>
-      <c r="E44" s="43"/>
+      <c r="C44" s="39"/>
+      <c r="D44" s="40"/>
+      <c r="E44" s="41"/>
       <c r="F44" s="25"/>
-      <c r="G44" s="56"/>
-      <c r="H44" s="56"/>
+      <c r="G44" s="54"/>
+      <c r="H44" s="54"/>
       <c r="J44" s="28"/>
     </row>
     <row r="45" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="24"/>
-      <c r="B45" s="44"/>
-      <c r="C45" s="41"/>
-      <c r="D45" s="42"/>
-      <c r="E45" s="43"/>
+      <c r="B45" s="42"/>
+      <c r="C45" s="39"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="41"/>
       <c r="F45" s="25"/>
       <c r="G45" s="24"/>
-      <c r="H45" s="56"/>
+      <c r="H45" s="54"/>
       <c r="J45" s="28"/>
     </row>
     <row r="46" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="24"/>
-      <c r="B46" s="71"/>
-      <c r="C46" s="72"/>
-      <c r="D46" s="54"/>
-      <c r="E46" s="55"/>
+      <c r="B46" s="69"/>
+      <c r="C46" s="70"/>
+      <c r="D46" s="52"/>
+      <c r="E46" s="53"/>
       <c r="F46" s="25"/>
       <c r="G46" s="24"/>
-      <c r="H46" s="56"/>
+      <c r="H46" s="54"/>
       <c r="J46" s="28"/>
     </row>
     <row r="47" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="24"/>
-      <c r="B47" s="71"/>
-      <c r="C47" s="74"/>
-      <c r="D47" s="75"/>
-      <c r="E47" s="76"/>
+      <c r="B47" s="69"/>
+      <c r="C47" s="72"/>
+      <c r="D47" s="73"/>
+      <c r="E47" s="74"/>
       <c r="F47" s="25"/>
       <c r="G47" s="24"/>
-      <c r="H47" s="56"/>
+      <c r="H47" s="54"/>
       <c r="J47" s="28"/>
     </row>
     <row r="48" spans="1:10" s="31" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="23"/>
       <c r="B48" s="29"/>
-      <c r="C48" s="87"/>
-      <c r="D48" s="88"/>
-      <c r="E48" s="89"/>
+      <c r="C48" s="84"/>
+      <c r="D48" s="85"/>
+      <c r="E48" s="86"/>
       <c r="F48" s="30"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="56"/>
+      <c r="G48" s="39"/>
+      <c r="H48" s="54"/>
     </row>
     <row r="49" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="15"/>
@@ -3194,14 +2535,14 @@
       <c r="C49" s="15"/>
       <c r="D49" s="15"/>
       <c r="E49" s="15"/>
-      <c r="F49" s="53">
-        <f>SUM(F20:F47)</f>
+      <c r="F49" s="51">
+        <f>SUM(F20:F48)</f>
         <v>1</v>
       </c>
-      <c r="G49" s="77" t="s">
+      <c r="G49" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="H49" s="52">
+      <c r="H49" s="50">
         <f>SUM(H20:H48)</f>
         <v>0</v>
       </c>
@@ -3213,10 +2554,10 @@
       <c r="D50" s="15"/>
       <c r="E50" s="15"/>
       <c r="F50" s="32"/>
-      <c r="G50" s="77" t="s">
+      <c r="G50" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="H50" s="52">
+      <c r="H50" s="50">
         <f>H49*0.07</f>
         <v>0</v>
       </c>
@@ -3228,10 +2569,10 @@
       <c r="D51" s="15"/>
       <c r="E51" s="15"/>
       <c r="F51" s="32"/>
-      <c r="G51" s="77" t="s">
+      <c r="G51" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="H51" s="52">
+      <c r="H51" s="50">
         <f>SUM(H49:H50)</f>
         <v>0</v>
       </c>
@@ -3243,11 +2584,8 @@
       <c r="D52" s="15"/>
       <c r="E52" s="15"/>
       <c r="F52" s="34"/>
-      <c r="G52" s="86" t="str">
-        <f>"("&amp;BAHTTEXT(H$51)&amp;")"</f>
-        <v>(ศูนย์บาทถ้วน)</v>
-      </c>
-      <c r="H52" s="86"/>
+      <c r="G52" s="83"/>
+      <c r="H52" s="83"/>
     </row>
     <row r="53" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="35"/>
@@ -3259,52 +2597,115 @@
       <c r="G53" s="38"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" s="35"/>
-      <c r="B54" s="37"/>
-      <c r="C54" s="37"/>
+      <c r="A54" s="91" t="s">
+        <v>40</v>
+      </c>
+      <c r="B54" s="90"/>
+      <c r="C54" s="90"/>
       <c r="D54" s="15"/>
       <c r="E54" s="15"/>
       <c r="F54" s="15"/>
       <c r="G54" s="15"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B55" s="39"/>
-      <c r="C55" s="17"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="17"/>
+      <c r="A55" s="90"/>
+      <c r="B55" s="90"/>
+      <c r="C55" s="90"/>
+      <c r="D55" s="92" t="s">
+        <v>39</v>
+      </c>
+      <c r="E55" s="93"/>
+      <c r="F55" s="98" t="s">
+        <v>41</v>
+      </c>
+      <c r="G55" s="98"/>
+      <c r="H55" s="98"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B56" s="40"/>
-      <c r="C56" s="17"/>
-      <c r="D56" s="17"/>
-      <c r="E56" s="17"/>
-      <c r="F56" s="17"/>
+      <c r="A56" s="90"/>
+      <c r="B56" s="90"/>
+      <c r="C56" s="90"/>
+      <c r="D56" s="93"/>
+      <c r="E56" s="93"/>
+      <c r="F56" s="98"/>
+      <c r="G56" s="98"/>
+      <c r="H56" s="98"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A57" s="90"/>
+      <c r="B57" s="90"/>
+      <c r="C57" s="90"/>
+      <c r="D57" s="93"/>
+      <c r="E57" s="93"/>
+      <c r="F57" s="98"/>
+      <c r="G57" s="98"/>
+      <c r="H57" s="98"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A58" s="39"/>
-      <c r="B58" s="39"/>
-      <c r="C58" s="39"/>
-      <c r="D58" s="39"/>
-      <c r="E58" s="39"/>
-      <c r="F58" s="39"/>
-      <c r="G58" s="39"/>
+      <c r="A58" s="90"/>
+      <c r="B58" s="90"/>
+      <c r="C58" s="90"/>
+      <c r="D58" s="93"/>
+      <c r="E58" s="93"/>
+      <c r="F58" s="98"/>
+      <c r="G58" s="98"/>
+      <c r="H58" s="98"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A59" s="90"/>
+      <c r="B59" s="90"/>
+      <c r="C59" s="90"/>
+      <c r="D59" s="93"/>
+      <c r="E59" s="93"/>
+      <c r="F59" s="98"/>
+      <c r="G59" s="98"/>
+      <c r="H59" s="98"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A60" s="90"/>
+      <c r="B60" s="90"/>
+      <c r="C60" s="90"/>
+      <c r="D60" s="93"/>
+      <c r="E60" s="93"/>
+      <c r="F60" s="98"/>
+      <c r="G60" s="98"/>
+      <c r="H60" s="98"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D61" s="85"/>
-      <c r="E61" s="85"/>
+      <c r="A61" s="90"/>
+      <c r="B61" s="90"/>
+      <c r="C61" s="90"/>
+      <c r="D61" s="93"/>
+      <c r="E61" s="93"/>
+      <c r="F61" s="98"/>
+      <c r="G61" s="98"/>
+      <c r="H61" s="98"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A62" s="90"/>
+      <c r="B62" s="90"/>
+      <c r="C62" s="90"/>
+      <c r="D62" s="93"/>
+      <c r="E62" s="93"/>
+      <c r="F62" s="98"/>
+      <c r="G62" s="98"/>
+      <c r="H62" s="98"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="13">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="G11:H12"/>
+    <mergeCell ref="F55:H62"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="F16:G16"/>
-    <mergeCell ref="D61:E61"/>
     <mergeCell ref="G52:H52"/>
     <mergeCell ref="C48:E48"/>
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="C19:E19"/>
+    <mergeCell ref="A54:C62"/>
+    <mergeCell ref="D55:E62"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H5:H6" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>